<commit_message>
Rotate resource enemies along orbit path
</commit_message>
<xml_diff>
--- a/Luban/Datas/WaveSpawn.xlsx
+++ b/Luban/Datas/WaveSpawn.xlsx
@@ -2484,602 +2484,602 @@
       </c>
     </row>
     <row r="36">
-      <c r="B36" t="n">
+      <c r="B36" s="0" t="n">
         <v>33</v>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_orbit_01</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D36" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_orbit</t>
         </is>
       </c>
-      <c r="E36" t="n">
-        <v>1</v>
-      </c>
-      <c r="F36" t="inlineStr">
+      <c r="E36" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G36" t="n">
-        <v>1</v>
-      </c>
-      <c r="H36" t="n">
+      <c r="G36" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H36" s="0" t="n">
         <v>0.1</v>
       </c>
-      <c r="I36" t="n">
+      <c r="I36" s="0" t="n">
         <v>-5.4</v>
       </c>
-      <c r="J36" t="n">
+      <c r="J36" s="0" t="n">
         <v>7.6</v>
       </c>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>Orbit:centerX=-0.45,centerY=2.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,exitDirection=DownRight,exitSpeed=3.4</t>
-        </is>
-      </c>
-      <c r="M36" t="n">
-        <v>0</v>
-      </c>
-      <c r="N36" t="n">
-        <v>0</v>
-      </c>
-      <c r="O36" t="n">
+      <c r="K36" s="0" t="inlineStr"/>
+      <c r="L36" s="0" t="inlineStr">
+        <is>
+          <t>Orbit:centerX=-0.45,centerY=2.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,exitDirection=DownRight,exitSpeed=3.4</t>
+        </is>
+      </c>
+      <c r="M36" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N36" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="37">
-      <c r="B37" t="n">
+      <c r="B37" s="0" t="n">
         <v>34</v>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_orbit_02</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_orbit</t>
         </is>
       </c>
-      <c r="E37" t="n">
+      <c r="E37" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F37" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G37" t="n">
-        <v>1</v>
-      </c>
-      <c r="H37" t="n">
+      <c r="G37" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H37" s="0" t="n">
         <v>0.1</v>
       </c>
-      <c r="I37" t="n">
+      <c r="I37" s="0" t="n">
         <v>-4.7</v>
       </c>
-      <c r="J37" t="n">
+      <c r="J37" s="0" t="n">
         <v>7.6</v>
       </c>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>Orbit:centerX=0.45,centerY=2.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,exitDirection=DownRight,exitSpeed=3.4</t>
-        </is>
-      </c>
-      <c r="M37" t="n">
-        <v>0</v>
-      </c>
-      <c r="N37" t="n">
-        <v>0</v>
-      </c>
-      <c r="O37" t="n">
+      <c r="K37" s="0" t="inlineStr"/>
+      <c r="L37" s="0" t="inlineStr">
+        <is>
+          <t>Orbit:centerX=0.45,centerY=2.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,exitDirection=DownRight,exitSpeed=3.4</t>
+        </is>
+      </c>
+      <c r="M37" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N37" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O37" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="38">
-      <c r="B38" t="n">
+      <c r="B38" s="0" t="n">
         <v>35</v>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C38" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_orbit_03</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D38" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_orbit</t>
         </is>
       </c>
-      <c r="E38" t="n">
+      <c r="E38" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="F38" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G38" t="n">
-        <v>1</v>
-      </c>
-      <c r="H38" t="n">
+      <c r="G38" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H38" s="0" t="n">
         <v>0.1</v>
       </c>
-      <c r="I38" t="n">
+      <c r="I38" s="0" t="n">
         <v>-5.4</v>
       </c>
-      <c r="J38" t="n">
+      <c r="J38" s="0" t="n">
         <v>7.1</v>
       </c>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>Orbit:centerX=-0.45,centerY=1.75,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,exitDirection=DownRight,exitSpeed=3.4</t>
-        </is>
-      </c>
-      <c r="M38" t="n">
-        <v>0</v>
-      </c>
-      <c r="N38" t="n">
-        <v>0</v>
-      </c>
-      <c r="O38" t="n">
+      <c r="K38" s="0" t="inlineStr"/>
+      <c r="L38" s="0" t="inlineStr">
+        <is>
+          <t>Orbit:centerX=-0.45,centerY=1.75,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,exitDirection=DownRight,exitSpeed=3.4</t>
+        </is>
+      </c>
+      <c r="M38" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N38" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O38" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="39">
-      <c r="B39" t="n">
+      <c r="B39" s="0" t="n">
         <v>36</v>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_orbit_04</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_orbit</t>
         </is>
       </c>
-      <c r="E39" t="n">
+      <c r="E39" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F39" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G39" t="n">
-        <v>1</v>
-      </c>
-      <c r="H39" t="n">
+      <c r="G39" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H39" s="0" t="n">
         <v>0.1</v>
       </c>
-      <c r="I39" t="n">
+      <c r="I39" s="0" t="n">
         <v>-4.7</v>
       </c>
-      <c r="J39" t="n">
+      <c r="J39" s="0" t="n">
         <v>7.1</v>
       </c>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr">
-        <is>
-          <t>Orbit:centerX=0.45,centerY=1.75,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,exitDirection=DownRight,exitSpeed=3.4</t>
-        </is>
-      </c>
-      <c r="M39" t="n">
-        <v>0</v>
-      </c>
-      <c r="N39" t="n">
-        <v>0</v>
-      </c>
-      <c r="O39" t="n">
+      <c r="K39" s="0" t="inlineStr"/>
+      <c r="L39" s="0" t="inlineStr">
+        <is>
+          <t>Orbit:centerX=0.45,centerY=1.75,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,exitDirection=DownRight,exitSpeed=3.4</t>
+        </is>
+      </c>
+      <c r="M39" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N39" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O39" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="40">
-      <c r="B40" t="n">
+      <c r="B40" s="0" t="n">
         <v>37</v>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_orbit_05</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D40" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_orbit</t>
         </is>
       </c>
-      <c r="E40" t="n">
+      <c r="E40" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F40" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G40" t="n">
-        <v>1</v>
-      </c>
-      <c r="H40" t="n">
+      <c r="G40" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H40" s="0" t="n">
         <v>0.1</v>
       </c>
-      <c r="I40" t="n">
+      <c r="I40" s="0" t="n">
         <v>-5.4</v>
       </c>
-      <c r="J40" t="n">
+      <c r="J40" s="0" t="n">
         <v>6.6</v>
       </c>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr">
-        <is>
-          <t>Orbit:centerX=-0.45,centerY=1.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,exitDirection=DownRight,exitSpeed=3.4</t>
-        </is>
-      </c>
-      <c r="M40" t="n">
-        <v>0</v>
-      </c>
-      <c r="N40" t="n">
-        <v>0</v>
-      </c>
-      <c r="O40" t="n">
+      <c r="K40" s="0" t="inlineStr"/>
+      <c r="L40" s="0" t="inlineStr">
+        <is>
+          <t>Orbit:centerX=-0.45,centerY=1.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,exitDirection=DownRight,exitSpeed=3.4</t>
+        </is>
+      </c>
+      <c r="M40" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N40" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O40" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="41">
-      <c r="B41" t="n">
+      <c r="B41" s="0" t="n">
         <v>38</v>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_orbit_06</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_orbit</t>
         </is>
       </c>
-      <c r="E41" t="n">
+      <c r="E41" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F41" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G41" t="n">
-        <v>1</v>
-      </c>
-      <c r="H41" t="n">
+      <c r="G41" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H41" s="0" t="n">
         <v>0.1</v>
       </c>
-      <c r="I41" t="n">
+      <c r="I41" s="0" t="n">
         <v>-4.7</v>
       </c>
-      <c r="J41" t="n">
+      <c r="J41" s="0" t="n">
         <v>6.6</v>
       </c>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>Orbit:centerX=0.45,centerY=1.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,exitDirection=DownRight,exitSpeed=3.4</t>
-        </is>
-      </c>
-      <c r="M41" t="n">
-        <v>0</v>
-      </c>
-      <c r="N41" t="n">
-        <v>0</v>
-      </c>
-      <c r="O41" t="n">
+      <c r="K41" s="0" t="inlineStr"/>
+      <c r="L41" s="0" t="inlineStr">
+        <is>
+          <t>Orbit:centerX=0.45,centerY=1.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,exitDirection=DownRight,exitSpeed=3.4</t>
+        </is>
+      </c>
+      <c r="M41" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N41" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O41" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="42">
-      <c r="B42" t="n">
+      <c r="B42" s="0" t="n">
         <v>39</v>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_orbit_07</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D42" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_orbit</t>
         </is>
       </c>
-      <c r="E42" t="n">
+      <c r="E42" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F42" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G42" t="n">
-        <v>1</v>
-      </c>
-      <c r="H42" t="n">
+      <c r="G42" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H42" s="0" t="n">
         <v>0.1</v>
       </c>
-      <c r="I42" t="n">
+      <c r="I42" s="0" t="n">
         <v>-5.4</v>
       </c>
-      <c r="J42" t="n">
+      <c r="J42" s="0" t="n">
         <v>6.1</v>
       </c>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>Orbit:centerX=-0.45,centerY=0.75,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,exitDirection=DownRight,exitSpeed=3.4</t>
-        </is>
-      </c>
-      <c r="M42" t="n">
-        <v>0</v>
-      </c>
-      <c r="N42" t="n">
-        <v>0</v>
-      </c>
-      <c r="O42" t="n">
+      <c r="K42" s="0" t="inlineStr"/>
+      <c r="L42" s="0" t="inlineStr">
+        <is>
+          <t>Orbit:centerX=-0.45,centerY=0.75,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,exitDirection=DownRight,exitSpeed=3.4</t>
+        </is>
+      </c>
+      <c r="M42" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N42" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O42" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="43">
-      <c r="B43" t="n">
+      <c r="B43" s="0" t="n">
         <v>40</v>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_orbit_08</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D43" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_orbit</t>
         </is>
       </c>
-      <c r="E43" t="n">
+      <c r="E43" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F43" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G43" t="n">
-        <v>1</v>
-      </c>
-      <c r="H43" t="n">
+      <c r="G43" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H43" s="0" t="n">
         <v>0.1</v>
       </c>
-      <c r="I43" t="n">
+      <c r="I43" s="0" t="n">
         <v>-4.7</v>
       </c>
-      <c r="J43" t="n">
+      <c r="J43" s="0" t="n">
         <v>6.1</v>
       </c>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>Orbit:centerX=0.45,centerY=0.75,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,exitDirection=DownRight,exitSpeed=3.4</t>
-        </is>
-      </c>
-      <c r="M43" t="n">
-        <v>0</v>
-      </c>
-      <c r="N43" t="n">
-        <v>0</v>
-      </c>
-      <c r="O43" t="n">
+      <c r="K43" s="0" t="inlineStr"/>
+      <c r="L43" s="0" t="inlineStr">
+        <is>
+          <t>Orbit:centerX=0.45,centerY=0.75,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,exitDirection=DownRight,exitSpeed=3.4</t>
+        </is>
+      </c>
+      <c r="M43" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N43" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O43" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="44">
-      <c r="B44" t="n">
+      <c r="B44" s="0" t="n">
         <v>41</v>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C44" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_orbit_09</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D44" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_orbit</t>
         </is>
       </c>
-      <c r="E44" t="n">
+      <c r="E44" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="F44" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G44" t="n">
-        <v>1</v>
-      </c>
-      <c r="H44" t="n">
+      <c r="G44" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H44" s="0" t="n">
         <v>0.1</v>
       </c>
-      <c r="I44" t="n">
+      <c r="I44" s="0" t="n">
         <v>-5.4</v>
       </c>
-      <c r="J44" t="n">
+      <c r="J44" s="0" t="n">
         <v>5.6</v>
       </c>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>Orbit:centerX=-0.45,centerY=0.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,exitDirection=DownRight,exitSpeed=3.4</t>
-        </is>
-      </c>
-      <c r="M44" t="n">
-        <v>0</v>
-      </c>
-      <c r="N44" t="n">
-        <v>0</v>
-      </c>
-      <c r="O44" t="n">
+      <c r="K44" s="0" t="inlineStr"/>
+      <c r="L44" s="0" t="inlineStr">
+        <is>
+          <t>Orbit:centerX=-0.45,centerY=0.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,exitDirection=DownRight,exitSpeed=3.4</t>
+        </is>
+      </c>
+      <c r="M44" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N44" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O44" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="45">
-      <c r="B45" t="n">
+      <c r="B45" s="0" t="n">
         <v>42</v>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_orbit_10</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_orbit</t>
         </is>
       </c>
-      <c r="E45" t="n">
+      <c r="E45" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F45" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G45" t="n">
-        <v>1</v>
-      </c>
-      <c r="H45" t="n">
+      <c r="G45" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H45" s="0" t="n">
         <v>0.1</v>
       </c>
-      <c r="I45" t="n">
+      <c r="I45" s="0" t="n">
         <v>-4.7</v>
       </c>
-      <c r="J45" t="n">
+      <c r="J45" s="0" t="n">
         <v>5.6</v>
       </c>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>Orbit:centerX=0.45,centerY=0.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,exitDirection=DownRight,exitSpeed=3.4</t>
-        </is>
-      </c>
-      <c r="M45" t="n">
-        <v>0</v>
-      </c>
-      <c r="N45" t="n">
-        <v>0</v>
-      </c>
-      <c r="O45" t="n">
+      <c r="K45" s="0" t="inlineStr"/>
+      <c r="L45" s="0" t="inlineStr">
+        <is>
+          <t>Orbit:centerX=0.45,centerY=0.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,exitDirection=DownRight,exitSpeed=3.4</t>
+        </is>
+      </c>
+      <c r="M45" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N45" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O45" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="46">
-      <c r="B46" t="n">
+      <c r="B46" s="0" t="n">
         <v>43</v>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_orbit_11</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D46" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_orbit</t>
         </is>
       </c>
-      <c r="E46" t="n">
+      <c r="E46" s="0" t="n">
         <v>11</v>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F46" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G46" t="n">
-        <v>1</v>
-      </c>
-      <c r="H46" t="n">
+      <c r="G46" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H46" s="0" t="n">
         <v>0.1</v>
       </c>
-      <c r="I46" t="n">
+      <c r="I46" s="0" t="n">
         <v>-5.4</v>
       </c>
-      <c r="J46" t="n">
+      <c r="J46" s="0" t="n">
         <v>5.1</v>
       </c>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>Orbit:centerX=-0.45,centerY=-0.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,exitDirection=DownRight,exitSpeed=3.4</t>
-        </is>
-      </c>
-      <c r="M46" t="n">
-        <v>0</v>
-      </c>
-      <c r="N46" t="n">
-        <v>0</v>
-      </c>
-      <c r="O46" t="n">
+      <c r="K46" s="0" t="inlineStr"/>
+      <c r="L46" s="0" t="inlineStr">
+        <is>
+          <t>Orbit:centerX=-0.45,centerY=-0.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,exitDirection=DownRight,exitSpeed=3.4</t>
+        </is>
+      </c>
+      <c r="M46" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N46" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O46" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="47">
-      <c r="B47" t="n">
+      <c r="B47" s="0" t="n">
         <v>44</v>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_orbit_12</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D47" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_orbit</t>
         </is>
       </c>
-      <c r="E47" t="n">
+      <c r="E47" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="F47" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G47" t="n">
-        <v>1</v>
-      </c>
-      <c r="H47" t="n">
+      <c r="G47" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H47" s="0" t="n">
         <v>0.1</v>
       </c>
-      <c r="I47" t="n">
+      <c r="I47" s="0" t="n">
         <v>-4.7</v>
       </c>
-      <c r="J47" t="n">
+      <c r="J47" s="0" t="n">
         <v>5.1</v>
       </c>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>Orbit:centerX=0.45,centerY=-0.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,exitDirection=DownRight,exitSpeed=3.4</t>
-        </is>
-      </c>
-      <c r="M47" t="n">
-        <v>0</v>
-      </c>
-      <c r="N47" t="n">
-        <v>0</v>
-      </c>
-      <c r="O47" t="n">
+      <c r="K47" s="0" t="inlineStr"/>
+      <c r="L47" s="0" t="inlineStr">
+        <is>
+          <t>Orbit:centerX=0.45,centerY=-0.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,exitDirection=DownRight,exitSpeed=3.4</t>
+        </is>
+      </c>
+      <c r="M47" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N47" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O47" s="0" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix resource enemy path rotation offset
</commit_message>
<xml_diff>
--- a/Luban/Datas/WaveSpawn.xlsx
+++ b/Luban/Datas/WaveSpawn.xlsx
@@ -2520,7 +2520,7 @@
       <c r="K36" s="0" t="inlineStr"/>
       <c r="L36" s="0" t="inlineStr">
         <is>
-          <t>Orbit:centerX=-0.45,centerY=2.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,exitDirection=DownRight,exitSpeed=3.4</t>
+          <t>Orbit:centerX=-0.45,centerY=2.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
         </is>
       </c>
       <c r="M36" s="0" t="n">
@@ -2570,7 +2570,7 @@
       <c r="K37" s="0" t="inlineStr"/>
       <c r="L37" s="0" t="inlineStr">
         <is>
-          <t>Orbit:centerX=0.45,centerY=2.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,exitDirection=DownRight,exitSpeed=3.4</t>
+          <t>Orbit:centerX=0.45,centerY=2.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
         </is>
       </c>
       <c r="M37" s="0" t="n">
@@ -2620,7 +2620,7 @@
       <c r="K38" s="0" t="inlineStr"/>
       <c r="L38" s="0" t="inlineStr">
         <is>
-          <t>Orbit:centerX=-0.45,centerY=1.75,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,exitDirection=DownRight,exitSpeed=3.4</t>
+          <t>Orbit:centerX=-0.45,centerY=1.75,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
         </is>
       </c>
       <c r="M38" s="0" t="n">
@@ -2670,7 +2670,7 @@
       <c r="K39" s="0" t="inlineStr"/>
       <c r="L39" s="0" t="inlineStr">
         <is>
-          <t>Orbit:centerX=0.45,centerY=1.75,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,exitDirection=DownRight,exitSpeed=3.4</t>
+          <t>Orbit:centerX=0.45,centerY=1.75,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
         </is>
       </c>
       <c r="M39" s="0" t="n">
@@ -2720,7 +2720,7 @@
       <c r="K40" s="0" t="inlineStr"/>
       <c r="L40" s="0" t="inlineStr">
         <is>
-          <t>Orbit:centerX=-0.45,centerY=1.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,exitDirection=DownRight,exitSpeed=3.4</t>
+          <t>Orbit:centerX=-0.45,centerY=1.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
         </is>
       </c>
       <c r="M40" s="0" t="n">
@@ -2770,7 +2770,7 @@
       <c r="K41" s="0" t="inlineStr"/>
       <c r="L41" s="0" t="inlineStr">
         <is>
-          <t>Orbit:centerX=0.45,centerY=1.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,exitDirection=DownRight,exitSpeed=3.4</t>
+          <t>Orbit:centerX=0.45,centerY=1.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
         </is>
       </c>
       <c r="M41" s="0" t="n">
@@ -2820,7 +2820,7 @@
       <c r="K42" s="0" t="inlineStr"/>
       <c r="L42" s="0" t="inlineStr">
         <is>
-          <t>Orbit:centerX=-0.45,centerY=0.75,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,exitDirection=DownRight,exitSpeed=3.4</t>
+          <t>Orbit:centerX=-0.45,centerY=0.75,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
         </is>
       </c>
       <c r="M42" s="0" t="n">
@@ -2870,7 +2870,7 @@
       <c r="K43" s="0" t="inlineStr"/>
       <c r="L43" s="0" t="inlineStr">
         <is>
-          <t>Orbit:centerX=0.45,centerY=0.75,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,exitDirection=DownRight,exitSpeed=3.4</t>
+          <t>Orbit:centerX=0.45,centerY=0.75,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
         </is>
       </c>
       <c r="M43" s="0" t="n">
@@ -2920,7 +2920,7 @@
       <c r="K44" s="0" t="inlineStr"/>
       <c r="L44" s="0" t="inlineStr">
         <is>
-          <t>Orbit:centerX=-0.45,centerY=0.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,exitDirection=DownRight,exitSpeed=3.4</t>
+          <t>Orbit:centerX=-0.45,centerY=0.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
         </is>
       </c>
       <c r="M44" s="0" t="n">
@@ -2970,7 +2970,7 @@
       <c r="K45" s="0" t="inlineStr"/>
       <c r="L45" s="0" t="inlineStr">
         <is>
-          <t>Orbit:centerX=0.45,centerY=0.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,exitDirection=DownRight,exitSpeed=3.4</t>
+          <t>Orbit:centerX=0.45,centerY=0.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
         </is>
       </c>
       <c r="M45" s="0" t="n">
@@ -3020,7 +3020,7 @@
       <c r="K46" s="0" t="inlineStr"/>
       <c r="L46" s="0" t="inlineStr">
         <is>
-          <t>Orbit:centerX=-0.45,centerY=-0.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,exitDirection=DownRight,exitSpeed=3.4</t>
+          <t>Orbit:centerX=-0.45,centerY=-0.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
         </is>
       </c>
       <c r="M46" s="0" t="n">
@@ -3070,7 +3070,7 @@
       <c r="K47" s="0" t="inlineStr"/>
       <c r="L47" s="0" t="inlineStr">
         <is>
-          <t>Orbit:centerX=0.45,centerY=-0.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,exitDirection=DownRight,exitSpeed=3.4</t>
+          <t>Orbit:centerX=0.45,centerY=-0.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
         </is>
       </c>
       <c r="M47" s="0" t="n">

</xml_diff>

<commit_message>
Increase resource enemy orbit radius
</commit_message>
<xml_diff>
--- a/Luban/Datas/WaveSpawn.xlsx
+++ b/Luban/Datas/WaveSpawn.xlsx
@@ -2520,7 +2520,7 @@
       <c r="K36" s="0" t="inlineStr"/>
       <c r="L36" s="0" t="inlineStr">
         <is>
-          <t>Orbit:centerX=-0.45,centerY=2.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
+          <t>Orbit:centerX=-0.45,centerY=2.25,radiusX=3.6,radiusY=3.6,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
         </is>
       </c>
       <c r="M36" s="0" t="n">
@@ -2570,7 +2570,7 @@
       <c r="K37" s="0" t="inlineStr"/>
       <c r="L37" s="0" t="inlineStr">
         <is>
-          <t>Orbit:centerX=0.45,centerY=2.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
+          <t>Orbit:centerX=0.45,centerY=2.25,radiusX=3.6,radiusY=3.6,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
         </is>
       </c>
       <c r="M37" s="0" t="n">
@@ -2620,7 +2620,7 @@
       <c r="K38" s="0" t="inlineStr"/>
       <c r="L38" s="0" t="inlineStr">
         <is>
-          <t>Orbit:centerX=-0.45,centerY=1.75,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
+          <t>Orbit:centerX=-0.45,centerY=1.75,radiusX=3.6,radiusY=3.6,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
         </is>
       </c>
       <c r="M38" s="0" t="n">
@@ -2670,7 +2670,7 @@
       <c r="K39" s="0" t="inlineStr"/>
       <c r="L39" s="0" t="inlineStr">
         <is>
-          <t>Orbit:centerX=0.45,centerY=1.75,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
+          <t>Orbit:centerX=0.45,centerY=1.75,radiusX=3.6,radiusY=3.6,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
         </is>
       </c>
       <c r="M39" s="0" t="n">
@@ -2720,7 +2720,7 @@
       <c r="K40" s="0" t="inlineStr"/>
       <c r="L40" s="0" t="inlineStr">
         <is>
-          <t>Orbit:centerX=-0.45,centerY=1.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
+          <t>Orbit:centerX=-0.45,centerY=1.25,radiusX=3.6,radiusY=3.6,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
         </is>
       </c>
       <c r="M40" s="0" t="n">
@@ -2770,7 +2770,7 @@
       <c r="K41" s="0" t="inlineStr"/>
       <c r="L41" s="0" t="inlineStr">
         <is>
-          <t>Orbit:centerX=0.45,centerY=1.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
+          <t>Orbit:centerX=0.45,centerY=1.25,radiusX=3.6,radiusY=3.6,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
         </is>
       </c>
       <c r="M41" s="0" t="n">
@@ -2820,7 +2820,7 @@
       <c r="K42" s="0" t="inlineStr"/>
       <c r="L42" s="0" t="inlineStr">
         <is>
-          <t>Orbit:centerX=-0.45,centerY=0.75,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
+          <t>Orbit:centerX=-0.45,centerY=0.75,radiusX=3.6,radiusY=3.6,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
         </is>
       </c>
       <c r="M42" s="0" t="n">
@@ -2870,7 +2870,7 @@
       <c r="K43" s="0" t="inlineStr"/>
       <c r="L43" s="0" t="inlineStr">
         <is>
-          <t>Orbit:centerX=0.45,centerY=0.75,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
+          <t>Orbit:centerX=0.45,centerY=0.75,radiusX=3.6,radiusY=3.6,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
         </is>
       </c>
       <c r="M43" s="0" t="n">
@@ -2920,7 +2920,7 @@
       <c r="K44" s="0" t="inlineStr"/>
       <c r="L44" s="0" t="inlineStr">
         <is>
-          <t>Orbit:centerX=-0.45,centerY=0.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
+          <t>Orbit:centerX=-0.45,centerY=0.25,radiusX=3.6,radiusY=3.6,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
         </is>
       </c>
       <c r="M44" s="0" t="n">
@@ -2970,7 +2970,7 @@
       <c r="K45" s="0" t="inlineStr"/>
       <c r="L45" s="0" t="inlineStr">
         <is>
-          <t>Orbit:centerX=0.45,centerY=0.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
+          <t>Orbit:centerX=0.45,centerY=0.25,radiusX=3.6,radiusY=3.6,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
         </is>
       </c>
       <c r="M45" s="0" t="n">
@@ -3020,7 +3020,7 @@
       <c r="K46" s="0" t="inlineStr"/>
       <c r="L46" s="0" t="inlineStr">
         <is>
-          <t>Orbit:centerX=-0.45,centerY=-0.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
+          <t>Orbit:centerX=-0.45,centerY=-0.25,radiusX=3.6,radiusY=3.6,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
         </is>
       </c>
       <c r="M46" s="0" t="n">
@@ -3070,7 +3070,7 @@
       <c r="K47" s="0" t="inlineStr"/>
       <c r="L47" s="0" t="inlineStr">
         <is>
-          <t>Orbit:centerX=0.45,centerY=-0.25,radiusX=0.22,radiusY=0.16,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
+          <t>Orbit:centerX=0.45,centerY=-0.25,radiusX=3.6,radiusY=3.6,angularSpeed=120,clockwise=false,startAngle=180,duration=0,loopCount=1,enterDuration=2.7,rotateToPath=true,rotationOffset=90,exitDirection=DownRight,exitSpeed=3.4</t>
         </is>
       </c>
       <c r="M47" s="0" t="n">

</xml_diff>

<commit_message>
Rotate diagonal resource waves along path
</commit_message>
<xml_diff>
--- a/Luban/Datas/WaveSpawn.xlsx
+++ b/Luban/Datas/WaveSpawn.xlsx
@@ -3084,1802 +3084,1802 @@
       </c>
     </row>
     <row r="48">
-      <c r="B48" t="n">
+      <c r="B48" s="0" t="n">
         <v>45</v>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C48" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_left_downright_01</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D48" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_left_downright</t>
         </is>
       </c>
-      <c r="E48" t="n">
-        <v>1</v>
-      </c>
-      <c r="F48" t="inlineStr">
+      <c r="E48" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F48" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G48" t="n">
-        <v>1</v>
-      </c>
-      <c r="H48" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I48" t="n">
+      <c r="G48" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H48" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I48" s="0" t="n">
         <v>-5.4</v>
       </c>
-      <c r="J48" t="n">
+      <c r="J48" s="0" t="n">
         <v>10.6</v>
       </c>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr">
-        <is>
-          <t>DriftRight</t>
-        </is>
-      </c>
-      <c r="M48" t="n">
-        <v>0</v>
-      </c>
-      <c r="N48" t="n">
+      <c r="K48" s="0" t="inlineStr"/>
+      <c r="L48" s="0" t="inlineStr">
+        <is>
+          <t>DriftRight:rotateToPath=true,rotationOffset=90</t>
+        </is>
+      </c>
+      <c r="M48" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N48" s="0" t="n">
         <v>2.4</v>
       </c>
-      <c r="O48" t="n">
+      <c r="O48" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="49">
-      <c r="B49" t="n">
+      <c r="B49" s="0" t="n">
         <v>46</v>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C49" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_left_downright_02</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D49" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_left_downright</t>
         </is>
       </c>
-      <c r="E49" t="n">
+      <c r="E49" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="F49" t="inlineStr">
+      <c r="F49" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G49" t="n">
-        <v>1</v>
-      </c>
-      <c r="H49" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I49" t="n">
+      <c r="G49" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H49" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I49" s="0" t="n">
         <v>-4</v>
       </c>
-      <c r="J49" t="n">
+      <c r="J49" s="0" t="n">
         <v>10.6</v>
       </c>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>DriftRight</t>
-        </is>
-      </c>
-      <c r="M49" t="n">
-        <v>0</v>
-      </c>
-      <c r="N49" t="n">
+      <c r="K49" s="0" t="inlineStr"/>
+      <c r="L49" s="0" t="inlineStr">
+        <is>
+          <t>DriftRight:rotateToPath=true,rotationOffset=90</t>
+        </is>
+      </c>
+      <c r="M49" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N49" s="0" t="n">
         <v>2.4</v>
       </c>
-      <c r="O49" t="n">
+      <c r="O49" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="50">
-      <c r="B50" t="n">
+      <c r="B50" s="0" t="n">
         <v>47</v>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C50" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_left_downright_03</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D50" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_left_downright</t>
         </is>
       </c>
-      <c r="E50" t="n">
+      <c r="E50" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="F50" t="inlineStr">
+      <c r="F50" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G50" t="n">
-        <v>1</v>
-      </c>
-      <c r="H50" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I50" t="n">
+      <c r="G50" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H50" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I50" s="0" t="n">
         <v>-5.4</v>
       </c>
-      <c r="J50" t="n">
+      <c r="J50" s="0" t="n">
         <v>9.6</v>
       </c>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>DriftRight</t>
-        </is>
-      </c>
-      <c r="M50" t="n">
-        <v>0</v>
-      </c>
-      <c r="N50" t="n">
+      <c r="K50" s="0" t="inlineStr"/>
+      <c r="L50" s="0" t="inlineStr">
+        <is>
+          <t>DriftRight:rotateToPath=true,rotationOffset=90</t>
+        </is>
+      </c>
+      <c r="M50" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N50" s="0" t="n">
         <v>2.4</v>
       </c>
-      <c r="O50" t="n">
+      <c r="O50" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="51">
-      <c r="B51" t="n">
+      <c r="B51" s="0" t="n">
         <v>48</v>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C51" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_left_downright_04</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D51" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_left_downright</t>
         </is>
       </c>
-      <c r="E51" t="n">
+      <c r="E51" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="F51" t="inlineStr">
+      <c r="F51" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G51" t="n">
-        <v>1</v>
-      </c>
-      <c r="H51" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I51" t="n">
+      <c r="G51" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H51" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I51" s="0" t="n">
         <v>-4</v>
       </c>
-      <c r="J51" t="n">
+      <c r="J51" s="0" t="n">
         <v>9.6</v>
       </c>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>DriftRight</t>
-        </is>
-      </c>
-      <c r="M51" t="n">
-        <v>0</v>
-      </c>
-      <c r="N51" t="n">
+      <c r="K51" s="0" t="inlineStr"/>
+      <c r="L51" s="0" t="inlineStr">
+        <is>
+          <t>DriftRight:rotateToPath=true,rotationOffset=90</t>
+        </is>
+      </c>
+      <c r="M51" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N51" s="0" t="n">
         <v>2.4</v>
       </c>
-      <c r="O51" t="n">
+      <c r="O51" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="52">
-      <c r="B52" t="n">
+      <c r="B52" s="0" t="n">
         <v>49</v>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C52" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_left_downright_05</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
+      <c r="D52" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_left_downright</t>
         </is>
       </c>
-      <c r="E52" t="n">
+      <c r="E52" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="F52" t="inlineStr">
+      <c r="F52" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G52" t="n">
-        <v>1</v>
-      </c>
-      <c r="H52" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I52" t="n">
+      <c r="G52" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H52" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I52" s="0" t="n">
         <v>-5.4</v>
       </c>
-      <c r="J52" t="n">
+      <c r="J52" s="0" t="n">
         <v>8.6</v>
       </c>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>DriftRight</t>
-        </is>
-      </c>
-      <c r="M52" t="n">
-        <v>0</v>
-      </c>
-      <c r="N52" t="n">
+      <c r="K52" s="0" t="inlineStr"/>
+      <c r="L52" s="0" t="inlineStr">
+        <is>
+          <t>DriftRight:rotateToPath=true,rotationOffset=90</t>
+        </is>
+      </c>
+      <c r="M52" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N52" s="0" t="n">
         <v>2.4</v>
       </c>
-      <c r="O52" t="n">
+      <c r="O52" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="53">
-      <c r="B53" t="n">
+      <c r="B53" s="0" t="n">
         <v>50</v>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C53" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_left_downright_06</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="D53" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_left_downright</t>
         </is>
       </c>
-      <c r="E53" t="n">
+      <c r="E53" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="F53" t="inlineStr">
+      <c r="F53" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G53" t="n">
-        <v>1</v>
-      </c>
-      <c r="H53" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I53" t="n">
+      <c r="G53" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H53" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I53" s="0" t="n">
         <v>-4</v>
       </c>
-      <c r="J53" t="n">
+      <c r="J53" s="0" t="n">
         <v>8.6</v>
       </c>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>DriftRight</t>
-        </is>
-      </c>
-      <c r="M53" t="n">
-        <v>0</v>
-      </c>
-      <c r="N53" t="n">
+      <c r="K53" s="0" t="inlineStr"/>
+      <c r="L53" s="0" t="inlineStr">
+        <is>
+          <t>DriftRight:rotateToPath=true,rotationOffset=90</t>
+        </is>
+      </c>
+      <c r="M53" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N53" s="0" t="n">
         <v>2.4</v>
       </c>
-      <c r="O53" t="n">
+      <c r="O53" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="54">
-      <c r="B54" t="n">
+      <c r="B54" s="0" t="n">
         <v>51</v>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C54" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_left_downright_07</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
+      <c r="D54" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_left_downright</t>
         </is>
       </c>
-      <c r="E54" t="n">
+      <c r="E54" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="F54" t="inlineStr">
+      <c r="F54" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G54" t="n">
-        <v>1</v>
-      </c>
-      <c r="H54" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I54" t="n">
+      <c r="G54" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H54" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I54" s="0" t="n">
         <v>-5.4</v>
       </c>
-      <c r="J54" t="n">
+      <c r="J54" s="0" t="n">
         <v>7.6</v>
       </c>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>DriftRight</t>
-        </is>
-      </c>
-      <c r="M54" t="n">
-        <v>0</v>
-      </c>
-      <c r="N54" t="n">
+      <c r="K54" s="0" t="inlineStr"/>
+      <c r="L54" s="0" t="inlineStr">
+        <is>
+          <t>DriftRight:rotateToPath=true,rotationOffset=90</t>
+        </is>
+      </c>
+      <c r="M54" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N54" s="0" t="n">
         <v>2.4</v>
       </c>
-      <c r="O54" t="n">
+      <c r="O54" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="55">
-      <c r="B55" t="n">
+      <c r="B55" s="0" t="n">
         <v>52</v>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C55" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_left_downright_08</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr">
+      <c r="D55" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_left_downright</t>
         </is>
       </c>
-      <c r="E55" t="n">
+      <c r="E55" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="F55" t="inlineStr">
+      <c r="F55" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G55" t="n">
-        <v>1</v>
-      </c>
-      <c r="H55" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I55" t="n">
+      <c r="G55" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H55" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I55" s="0" t="n">
         <v>-4</v>
       </c>
-      <c r="J55" t="n">
+      <c r="J55" s="0" t="n">
         <v>7.6</v>
       </c>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t>DriftRight</t>
-        </is>
-      </c>
-      <c r="M55" t="n">
-        <v>0</v>
-      </c>
-      <c r="N55" t="n">
+      <c r="K55" s="0" t="inlineStr"/>
+      <c r="L55" s="0" t="inlineStr">
+        <is>
+          <t>DriftRight:rotateToPath=true,rotationOffset=90</t>
+        </is>
+      </c>
+      <c r="M55" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N55" s="0" t="n">
         <v>2.4</v>
       </c>
-      <c r="O55" t="n">
+      <c r="O55" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="56">
-      <c r="B56" t="n">
+      <c r="B56" s="0" t="n">
         <v>53</v>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="C56" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_left_downright_09</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr">
+      <c r="D56" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_left_downright</t>
         </is>
       </c>
-      <c r="E56" t="n">
+      <c r="E56" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="F56" t="inlineStr">
+      <c r="F56" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G56" t="n">
-        <v>1</v>
-      </c>
-      <c r="H56" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I56" t="n">
+      <c r="G56" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H56" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I56" s="0" t="n">
         <v>-5.4</v>
       </c>
-      <c r="J56" t="n">
+      <c r="J56" s="0" t="n">
         <v>6.6</v>
       </c>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr">
-        <is>
-          <t>DriftRight</t>
-        </is>
-      </c>
-      <c r="M56" t="n">
-        <v>0</v>
-      </c>
-      <c r="N56" t="n">
+      <c r="K56" s="0" t="inlineStr"/>
+      <c r="L56" s="0" t="inlineStr">
+        <is>
+          <t>DriftRight:rotateToPath=true,rotationOffset=90</t>
+        </is>
+      </c>
+      <c r="M56" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N56" s="0" t="n">
         <v>2.4</v>
       </c>
-      <c r="O56" t="n">
+      <c r="O56" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="57">
-      <c r="B57" t="n">
+      <c r="B57" s="0" t="n">
         <v>54</v>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C57" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_left_downright_10</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
+      <c r="D57" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_left_downright</t>
         </is>
       </c>
-      <c r="E57" t="n">
+      <c r="E57" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="F57" t="inlineStr">
+      <c r="F57" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G57" t="n">
-        <v>1</v>
-      </c>
-      <c r="H57" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I57" t="n">
+      <c r="G57" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H57" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I57" s="0" t="n">
         <v>-4</v>
       </c>
-      <c r="J57" t="n">
+      <c r="J57" s="0" t="n">
         <v>6.6</v>
       </c>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr">
-        <is>
-          <t>DriftRight</t>
-        </is>
-      </c>
-      <c r="M57" t="n">
-        <v>0</v>
-      </c>
-      <c r="N57" t="n">
+      <c r="K57" s="0" t="inlineStr"/>
+      <c r="L57" s="0" t="inlineStr">
+        <is>
+          <t>DriftRight:rotateToPath=true,rotationOffset=90</t>
+        </is>
+      </c>
+      <c r="M57" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N57" s="0" t="n">
         <v>2.4</v>
       </c>
-      <c r="O57" t="n">
+      <c r="O57" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="58">
-      <c r="B58" t="n">
+      <c r="B58" s="0" t="n">
         <v>55</v>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C58" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_left_downright_11</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr">
+      <c r="D58" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_left_downright</t>
         </is>
       </c>
-      <c r="E58" t="n">
+      <c r="E58" s="0" t="n">
         <v>11</v>
       </c>
-      <c r="F58" t="inlineStr">
+      <c r="F58" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G58" t="n">
-        <v>1</v>
-      </c>
-      <c r="H58" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I58" t="n">
+      <c r="G58" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H58" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I58" s="0" t="n">
         <v>-5.4</v>
       </c>
-      <c r="J58" t="n">
+      <c r="J58" s="0" t="n">
         <v>5.6</v>
       </c>
-      <c r="K58" t="inlineStr"/>
-      <c r="L58" t="inlineStr">
-        <is>
-          <t>DriftRight</t>
-        </is>
-      </c>
-      <c r="M58" t="n">
-        <v>0</v>
-      </c>
-      <c r="N58" t="n">
+      <c r="K58" s="0" t="inlineStr"/>
+      <c r="L58" s="0" t="inlineStr">
+        <is>
+          <t>DriftRight:rotateToPath=true,rotationOffset=90</t>
+        </is>
+      </c>
+      <c r="M58" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N58" s="0" t="n">
         <v>2.4</v>
       </c>
-      <c r="O58" t="n">
+      <c r="O58" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="59">
-      <c r="B59" t="n">
+      <c r="B59" s="0" t="n">
         <v>56</v>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C59" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_left_downright_12</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr">
+      <c r="D59" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_left_downright</t>
         </is>
       </c>
-      <c r="E59" t="n">
+      <c r="E59" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="F59" t="inlineStr">
+      <c r="F59" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G59" t="n">
-        <v>1</v>
-      </c>
-      <c r="H59" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I59" t="n">
+      <c r="G59" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H59" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I59" s="0" t="n">
         <v>-4</v>
       </c>
-      <c r="J59" t="n">
+      <c r="J59" s="0" t="n">
         <v>5.6</v>
       </c>
-      <c r="K59" t="inlineStr"/>
-      <c r="L59" t="inlineStr">
-        <is>
-          <t>DriftRight</t>
-        </is>
-      </c>
-      <c r="M59" t="n">
-        <v>0</v>
-      </c>
-      <c r="N59" t="n">
+      <c r="K59" s="0" t="inlineStr"/>
+      <c r="L59" s="0" t="inlineStr">
+        <is>
+          <t>DriftRight:rotateToPath=true,rotationOffset=90</t>
+        </is>
+      </c>
+      <c r="M59" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N59" s="0" t="n">
         <v>2.4</v>
       </c>
-      <c r="O59" t="n">
+      <c r="O59" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="60">
-      <c r="B60" t="n">
+      <c r="B60" s="0" t="n">
         <v>57</v>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="C60" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_right_downleft_01</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr">
+      <c r="D60" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_right_downleft</t>
         </is>
       </c>
-      <c r="E60" t="n">
-        <v>1</v>
-      </c>
-      <c r="F60" t="inlineStr">
+      <c r="E60" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F60" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G60" t="n">
-        <v>1</v>
-      </c>
-      <c r="H60" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I60" t="n">
+      <c r="G60" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H60" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I60" s="0" t="n">
         <v>5.4</v>
       </c>
-      <c r="J60" t="n">
+      <c r="J60" s="0" t="n">
         <v>10.6</v>
       </c>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr">
-        <is>
-          <t>DriftLeft</t>
-        </is>
-      </c>
-      <c r="M60" t="n">
-        <v>0</v>
-      </c>
-      <c r="N60" t="n">
+      <c r="K60" s="0" t="inlineStr"/>
+      <c r="L60" s="0" t="inlineStr">
+        <is>
+          <t>DriftLeft:rotateToPath=true,rotationOffset=90</t>
+        </is>
+      </c>
+      <c r="M60" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N60" s="0" t="n">
         <v>2.4</v>
       </c>
-      <c r="O60" t="n">
+      <c r="O60" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="61">
-      <c r="B61" t="n">
+      <c r="B61" s="0" t="n">
         <v>58</v>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C61" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_right_downleft_02</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr">
+      <c r="D61" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_right_downleft</t>
         </is>
       </c>
-      <c r="E61" t="n">
+      <c r="E61" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="F61" t="inlineStr">
+      <c r="F61" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G61" t="n">
-        <v>1</v>
-      </c>
-      <c r="H61" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I61" t="n">
+      <c r="G61" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H61" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I61" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="J61" t="n">
+      <c r="J61" s="0" t="n">
         <v>10.6</v>
       </c>
-      <c r="K61" t="inlineStr"/>
-      <c r="L61" t="inlineStr">
-        <is>
-          <t>DriftLeft</t>
-        </is>
-      </c>
-      <c r="M61" t="n">
-        <v>0</v>
-      </c>
-      <c r="N61" t="n">
+      <c r="K61" s="0" t="inlineStr"/>
+      <c r="L61" s="0" t="inlineStr">
+        <is>
+          <t>DriftLeft:rotateToPath=true,rotationOffset=90</t>
+        </is>
+      </c>
+      <c r="M61" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N61" s="0" t="n">
         <v>2.4</v>
       </c>
-      <c r="O61" t="n">
+      <c r="O61" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="62">
-      <c r="B62" t="n">
+      <c r="B62" s="0" t="n">
         <v>59</v>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C62" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_right_downleft_03</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr">
+      <c r="D62" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_right_downleft</t>
         </is>
       </c>
-      <c r="E62" t="n">
+      <c r="E62" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="F62" t="inlineStr">
+      <c r="F62" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G62" t="n">
-        <v>1</v>
-      </c>
-      <c r="H62" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I62" t="n">
+      <c r="G62" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H62" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I62" s="0" t="n">
         <v>5.4</v>
       </c>
-      <c r="J62" t="n">
+      <c r="J62" s="0" t="n">
         <v>9.6</v>
       </c>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr">
-        <is>
-          <t>DriftLeft</t>
-        </is>
-      </c>
-      <c r="M62" t="n">
-        <v>0</v>
-      </c>
-      <c r="N62" t="n">
+      <c r="K62" s="0" t="inlineStr"/>
+      <c r="L62" s="0" t="inlineStr">
+        <is>
+          <t>DriftLeft:rotateToPath=true,rotationOffset=90</t>
+        </is>
+      </c>
+      <c r="M62" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N62" s="0" t="n">
         <v>2.4</v>
       </c>
-      <c r="O62" t="n">
+      <c r="O62" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="63">
-      <c r="B63" t="n">
+      <c r="B63" s="0" t="n">
         <v>60</v>
       </c>
-      <c r="C63" t="inlineStr">
+      <c r="C63" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_right_downleft_04</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr">
+      <c r="D63" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_right_downleft</t>
         </is>
       </c>
-      <c r="E63" t="n">
+      <c r="E63" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="F63" t="inlineStr">
+      <c r="F63" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G63" t="n">
-        <v>1</v>
-      </c>
-      <c r="H63" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I63" t="n">
+      <c r="G63" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H63" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I63" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="J63" t="n">
+      <c r="J63" s="0" t="n">
         <v>9.6</v>
       </c>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="inlineStr">
-        <is>
-          <t>DriftLeft</t>
-        </is>
-      </c>
-      <c r="M63" t="n">
-        <v>0</v>
-      </c>
-      <c r="N63" t="n">
+      <c r="K63" s="0" t="inlineStr"/>
+      <c r="L63" s="0" t="inlineStr">
+        <is>
+          <t>DriftLeft:rotateToPath=true,rotationOffset=90</t>
+        </is>
+      </c>
+      <c r="M63" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N63" s="0" t="n">
         <v>2.4</v>
       </c>
-      <c r="O63" t="n">
+      <c r="O63" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="64">
-      <c r="B64" t="n">
+      <c r="B64" s="0" t="n">
         <v>61</v>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C64" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_right_downleft_05</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr">
+      <c r="D64" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_right_downleft</t>
         </is>
       </c>
-      <c r="E64" t="n">
+      <c r="E64" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="F64" t="inlineStr">
+      <c r="F64" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G64" t="n">
-        <v>1</v>
-      </c>
-      <c r="H64" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I64" t="n">
+      <c r="G64" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H64" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I64" s="0" t="n">
         <v>5.4</v>
       </c>
-      <c r="J64" t="n">
+      <c r="J64" s="0" t="n">
         <v>8.6</v>
       </c>
-      <c r="K64" t="inlineStr"/>
-      <c r="L64" t="inlineStr">
-        <is>
-          <t>DriftLeft</t>
-        </is>
-      </c>
-      <c r="M64" t="n">
-        <v>0</v>
-      </c>
-      <c r="N64" t="n">
+      <c r="K64" s="0" t="inlineStr"/>
+      <c r="L64" s="0" t="inlineStr">
+        <is>
+          <t>DriftLeft:rotateToPath=true,rotationOffset=90</t>
+        </is>
+      </c>
+      <c r="M64" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N64" s="0" t="n">
         <v>2.4</v>
       </c>
-      <c r="O64" t="n">
+      <c r="O64" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="65">
-      <c r="B65" t="n">
+      <c r="B65" s="0" t="n">
         <v>62</v>
       </c>
-      <c r="C65" t="inlineStr">
+      <c r="C65" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_right_downleft_06</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr">
+      <c r="D65" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_right_downleft</t>
         </is>
       </c>
-      <c r="E65" t="n">
+      <c r="E65" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="F65" t="inlineStr">
+      <c r="F65" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G65" t="n">
-        <v>1</v>
-      </c>
-      <c r="H65" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I65" t="n">
+      <c r="G65" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H65" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I65" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="J65" t="n">
+      <c r="J65" s="0" t="n">
         <v>8.6</v>
       </c>
-      <c r="K65" t="inlineStr"/>
-      <c r="L65" t="inlineStr">
-        <is>
-          <t>DriftLeft</t>
-        </is>
-      </c>
-      <c r="M65" t="n">
-        <v>0</v>
-      </c>
-      <c r="N65" t="n">
+      <c r="K65" s="0" t="inlineStr"/>
+      <c r="L65" s="0" t="inlineStr">
+        <is>
+          <t>DriftLeft:rotateToPath=true,rotationOffset=90</t>
+        </is>
+      </c>
+      <c r="M65" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N65" s="0" t="n">
         <v>2.4</v>
       </c>
-      <c r="O65" t="n">
+      <c r="O65" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="66">
-      <c r="B66" t="n">
+      <c r="B66" s="0" t="n">
         <v>63</v>
       </c>
-      <c r="C66" t="inlineStr">
+      <c r="C66" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_right_downleft_07</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr">
+      <c r="D66" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_right_downleft</t>
         </is>
       </c>
-      <c r="E66" t="n">
+      <c r="E66" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="F66" t="inlineStr">
+      <c r="F66" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G66" t="n">
-        <v>1</v>
-      </c>
-      <c r="H66" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I66" t="n">
+      <c r="G66" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H66" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I66" s="0" t="n">
         <v>5.4</v>
       </c>
-      <c r="J66" t="n">
+      <c r="J66" s="0" t="n">
         <v>7.6</v>
       </c>
-      <c r="K66" t="inlineStr"/>
-      <c r="L66" t="inlineStr">
-        <is>
-          <t>DriftLeft</t>
-        </is>
-      </c>
-      <c r="M66" t="n">
-        <v>0</v>
-      </c>
-      <c r="N66" t="n">
+      <c r="K66" s="0" t="inlineStr"/>
+      <c r="L66" s="0" t="inlineStr">
+        <is>
+          <t>DriftLeft:rotateToPath=true,rotationOffset=90</t>
+        </is>
+      </c>
+      <c r="M66" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N66" s="0" t="n">
         <v>2.4</v>
       </c>
-      <c r="O66" t="n">
+      <c r="O66" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="67">
-      <c r="B67" t="n">
+      <c r="B67" s="0" t="n">
         <v>64</v>
       </c>
-      <c r="C67" t="inlineStr">
+      <c r="C67" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_right_downleft_08</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr">
+      <c r="D67" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_right_downleft</t>
         </is>
       </c>
-      <c r="E67" t="n">
+      <c r="E67" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="F67" t="inlineStr">
+      <c r="F67" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G67" t="n">
-        <v>1</v>
-      </c>
-      <c r="H67" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I67" t="n">
+      <c r="G67" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H67" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I67" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="J67" t="n">
+      <c r="J67" s="0" t="n">
         <v>7.6</v>
       </c>
-      <c r="K67" t="inlineStr"/>
-      <c r="L67" t="inlineStr">
-        <is>
-          <t>DriftLeft</t>
-        </is>
-      </c>
-      <c r="M67" t="n">
-        <v>0</v>
-      </c>
-      <c r="N67" t="n">
+      <c r="K67" s="0" t="inlineStr"/>
+      <c r="L67" s="0" t="inlineStr">
+        <is>
+          <t>DriftLeft:rotateToPath=true,rotationOffset=90</t>
+        </is>
+      </c>
+      <c r="M67" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N67" s="0" t="n">
         <v>2.4</v>
       </c>
-      <c r="O67" t="n">
+      <c r="O67" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="68">
-      <c r="B68" t="n">
+      <c r="B68" s="0" t="n">
         <v>65</v>
       </c>
-      <c r="C68" t="inlineStr">
+      <c r="C68" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_right_downleft_09</t>
         </is>
       </c>
-      <c r="D68" t="inlineStr">
+      <c r="D68" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_right_downleft</t>
         </is>
       </c>
-      <c r="E68" t="n">
+      <c r="E68" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="F68" t="inlineStr">
+      <c r="F68" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G68" t="n">
-        <v>1</v>
-      </c>
-      <c r="H68" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I68" t="n">
+      <c r="G68" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H68" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I68" s="0" t="n">
         <v>5.4</v>
       </c>
-      <c r="J68" t="n">
+      <c r="J68" s="0" t="n">
         <v>6.6</v>
       </c>
-      <c r="K68" t="inlineStr"/>
-      <c r="L68" t="inlineStr">
-        <is>
-          <t>DriftLeft</t>
-        </is>
-      </c>
-      <c r="M68" t="n">
-        <v>0</v>
-      </c>
-      <c r="N68" t="n">
+      <c r="K68" s="0" t="inlineStr"/>
+      <c r="L68" s="0" t="inlineStr">
+        <is>
+          <t>DriftLeft:rotateToPath=true,rotationOffset=90</t>
+        </is>
+      </c>
+      <c r="M68" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N68" s="0" t="n">
         <v>2.4</v>
       </c>
-      <c r="O68" t="n">
+      <c r="O68" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="69">
-      <c r="B69" t="n">
+      <c r="B69" s="0" t="n">
         <v>66</v>
       </c>
-      <c r="C69" t="inlineStr">
+      <c r="C69" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_right_downleft_10</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr">
+      <c r="D69" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_right_downleft</t>
         </is>
       </c>
-      <c r="E69" t="n">
+      <c r="E69" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="F69" t="inlineStr">
+      <c r="F69" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G69" t="n">
-        <v>1</v>
-      </c>
-      <c r="H69" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I69" t="n">
+      <c r="G69" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H69" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I69" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="J69" t="n">
+      <c r="J69" s="0" t="n">
         <v>6.6</v>
       </c>
-      <c r="K69" t="inlineStr"/>
-      <c r="L69" t="inlineStr">
-        <is>
-          <t>DriftLeft</t>
-        </is>
-      </c>
-      <c r="M69" t="n">
-        <v>0</v>
-      </c>
-      <c r="N69" t="n">
+      <c r="K69" s="0" t="inlineStr"/>
+      <c r="L69" s="0" t="inlineStr">
+        <is>
+          <t>DriftLeft:rotateToPath=true,rotationOffset=90</t>
+        </is>
+      </c>
+      <c r="M69" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N69" s="0" t="n">
         <v>2.4</v>
       </c>
-      <c r="O69" t="n">
+      <c r="O69" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="70">
-      <c r="B70" t="n">
+      <c r="B70" s="0" t="n">
         <v>67</v>
       </c>
-      <c r="C70" t="inlineStr">
+      <c r="C70" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_right_downleft_11</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr">
+      <c r="D70" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_right_downleft</t>
         </is>
       </c>
-      <c r="E70" t="n">
+      <c r="E70" s="0" t="n">
         <v>11</v>
       </c>
-      <c r="F70" t="inlineStr">
+      <c r="F70" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G70" t="n">
-        <v>1</v>
-      </c>
-      <c r="H70" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I70" t="n">
+      <c r="G70" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H70" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I70" s="0" t="n">
         <v>5.4</v>
       </c>
-      <c r="J70" t="n">
+      <c r="J70" s="0" t="n">
         <v>5.6</v>
       </c>
-      <c r="K70" t="inlineStr"/>
-      <c r="L70" t="inlineStr">
-        <is>
-          <t>DriftLeft</t>
-        </is>
-      </c>
-      <c r="M70" t="n">
-        <v>0</v>
-      </c>
-      <c r="N70" t="n">
+      <c r="K70" s="0" t="inlineStr"/>
+      <c r="L70" s="0" t="inlineStr">
+        <is>
+          <t>DriftLeft:rotateToPath=true,rotationOffset=90</t>
+        </is>
+      </c>
+      <c r="M70" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N70" s="0" t="n">
         <v>2.4</v>
       </c>
-      <c r="O70" t="n">
+      <c r="O70" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="71">
-      <c r="B71" t="n">
+      <c r="B71" s="0" t="n">
         <v>68</v>
       </c>
-      <c r="C71" t="inlineStr">
+      <c r="C71" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_right_downleft_12</t>
         </is>
       </c>
-      <c r="D71" t="inlineStr">
+      <c r="D71" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_right_downleft</t>
         </is>
       </c>
-      <c r="E71" t="n">
+      <c r="E71" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="F71" t="inlineStr">
+      <c r="F71" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G71" t="n">
-        <v>1</v>
-      </c>
-      <c r="H71" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I71" t="n">
+      <c r="G71" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H71" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I71" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="J71" t="n">
+      <c r="J71" s="0" t="n">
         <v>5.6</v>
       </c>
-      <c r="K71" t="inlineStr"/>
-      <c r="L71" t="inlineStr">
-        <is>
-          <t>DriftLeft</t>
-        </is>
-      </c>
-      <c r="M71" t="n">
-        <v>0</v>
-      </c>
-      <c r="N71" t="n">
+      <c r="K71" s="0" t="inlineStr"/>
+      <c r="L71" s="0" t="inlineStr">
+        <is>
+          <t>DriftLeft:rotateToPath=true,rotationOffset=90</t>
+        </is>
+      </c>
+      <c r="M71" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N71" s="0" t="n">
         <v>2.4</v>
       </c>
-      <c r="O71" t="n">
+      <c r="O71" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="72">
-      <c r="B72" t="n">
+      <c r="B72" s="0" t="n">
         <v>69</v>
       </c>
-      <c r="C72" t="inlineStr">
+      <c r="C72" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_top_down_01</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr">
+      <c r="D72" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_top_down</t>
         </is>
       </c>
-      <c r="E72" t="n">
-        <v>1</v>
-      </c>
-      <c r="F72" t="inlineStr">
+      <c r="E72" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F72" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G72" t="n">
-        <v>1</v>
-      </c>
-      <c r="H72" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I72" t="n">
+      <c r="G72" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H72" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I72" s="0" t="n">
         <v>-0.7</v>
       </c>
-      <c r="J72" t="n">
+      <c r="J72" s="0" t="n">
         <v>10.6</v>
       </c>
-      <c r="K72" t="inlineStr"/>
-      <c r="L72" t="inlineStr">
+      <c r="K72" s="0" t="inlineStr"/>
+      <c r="L72" s="0" t="inlineStr">
         <is>
           <t>Straight</t>
         </is>
       </c>
-      <c r="M72" t="n">
-        <v>0</v>
-      </c>
-      <c r="N72" t="n">
-        <v>0</v>
-      </c>
-      <c r="O72" t="n">
+      <c r="M72" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N72" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O72" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="73">
-      <c r="B73" t="n">
+      <c r="B73" s="0" t="n">
         <v>70</v>
       </c>
-      <c r="C73" t="inlineStr">
+      <c r="C73" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_top_down_02</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr">
+      <c r="D73" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_top_down</t>
         </is>
       </c>
-      <c r="E73" t="n">
+      <c r="E73" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="F73" t="inlineStr">
+      <c r="F73" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G73" t="n">
-        <v>1</v>
-      </c>
-      <c r="H73" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I73" t="n">
+      <c r="G73" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H73" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I73" s="0" t="n">
         <v>0.7</v>
       </c>
-      <c r="J73" t="n">
+      <c r="J73" s="0" t="n">
         <v>10.6</v>
       </c>
-      <c r="K73" t="inlineStr"/>
-      <c r="L73" t="inlineStr">
+      <c r="K73" s="0" t="inlineStr"/>
+      <c r="L73" s="0" t="inlineStr">
         <is>
           <t>Straight</t>
         </is>
       </c>
-      <c r="M73" t="n">
-        <v>0</v>
-      </c>
-      <c r="N73" t="n">
-        <v>0</v>
-      </c>
-      <c r="O73" t="n">
+      <c r="M73" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N73" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O73" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="74">
-      <c r="B74" t="n">
+      <c r="B74" s="0" t="n">
         <v>71</v>
       </c>
-      <c r="C74" t="inlineStr">
+      <c r="C74" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_top_down_03</t>
         </is>
       </c>
-      <c r="D74" t="inlineStr">
+      <c r="D74" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_top_down</t>
         </is>
       </c>
-      <c r="E74" t="n">
+      <c r="E74" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="F74" t="inlineStr">
+      <c r="F74" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G74" t="n">
-        <v>1</v>
-      </c>
-      <c r="H74" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I74" t="n">
+      <c r="G74" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H74" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I74" s="0" t="n">
         <v>-0.7</v>
       </c>
-      <c r="J74" t="n">
+      <c r="J74" s="0" t="n">
         <v>9.6</v>
       </c>
-      <c r="K74" t="inlineStr"/>
-      <c r="L74" t="inlineStr">
+      <c r="K74" s="0" t="inlineStr"/>
+      <c r="L74" s="0" t="inlineStr">
         <is>
           <t>Straight</t>
         </is>
       </c>
-      <c r="M74" t="n">
-        <v>0</v>
-      </c>
-      <c r="N74" t="n">
-        <v>0</v>
-      </c>
-      <c r="O74" t="n">
+      <c r="M74" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N74" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O74" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="75">
-      <c r="B75" t="n">
+      <c r="B75" s="0" t="n">
         <v>72</v>
       </c>
-      <c r="C75" t="inlineStr">
+      <c r="C75" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_top_down_04</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr">
+      <c r="D75" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_top_down</t>
         </is>
       </c>
-      <c r="E75" t="n">
+      <c r="E75" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="F75" t="inlineStr">
+      <c r="F75" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G75" t="n">
-        <v>1</v>
-      </c>
-      <c r="H75" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I75" t="n">
+      <c r="G75" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H75" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I75" s="0" t="n">
         <v>0.7</v>
       </c>
-      <c r="J75" t="n">
+      <c r="J75" s="0" t="n">
         <v>9.6</v>
       </c>
-      <c r="K75" t="inlineStr"/>
-      <c r="L75" t="inlineStr">
+      <c r="K75" s="0" t="inlineStr"/>
+      <c r="L75" s="0" t="inlineStr">
         <is>
           <t>Straight</t>
         </is>
       </c>
-      <c r="M75" t="n">
-        <v>0</v>
-      </c>
-      <c r="N75" t="n">
-        <v>0</v>
-      </c>
-      <c r="O75" t="n">
+      <c r="M75" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N75" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O75" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="76">
-      <c r="B76" t="n">
+      <c r="B76" s="0" t="n">
         <v>73</v>
       </c>
-      <c r="C76" t="inlineStr">
+      <c r="C76" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_top_down_05</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr">
+      <c r="D76" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_top_down</t>
         </is>
       </c>
-      <c r="E76" t="n">
+      <c r="E76" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="F76" t="inlineStr">
+      <c r="F76" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G76" t="n">
-        <v>1</v>
-      </c>
-      <c r="H76" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I76" t="n">
+      <c r="G76" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H76" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I76" s="0" t="n">
         <v>-0.7</v>
       </c>
-      <c r="J76" t="n">
+      <c r="J76" s="0" t="n">
         <v>8.6</v>
       </c>
-      <c r="K76" t="inlineStr"/>
-      <c r="L76" t="inlineStr">
+      <c r="K76" s="0" t="inlineStr"/>
+      <c r="L76" s="0" t="inlineStr">
         <is>
           <t>Straight</t>
         </is>
       </c>
-      <c r="M76" t="n">
-        <v>0</v>
-      </c>
-      <c r="N76" t="n">
-        <v>0</v>
-      </c>
-      <c r="O76" t="n">
+      <c r="M76" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N76" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O76" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="77">
-      <c r="B77" t="n">
+      <c r="B77" s="0" t="n">
         <v>74</v>
       </c>
-      <c r="C77" t="inlineStr">
+      <c r="C77" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_top_down_06</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr">
+      <c r="D77" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_top_down</t>
         </is>
       </c>
-      <c r="E77" t="n">
+      <c r="E77" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="F77" t="inlineStr">
+      <c r="F77" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G77" t="n">
-        <v>1</v>
-      </c>
-      <c r="H77" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I77" t="n">
+      <c r="G77" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H77" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I77" s="0" t="n">
         <v>0.7</v>
       </c>
-      <c r="J77" t="n">
+      <c r="J77" s="0" t="n">
         <v>8.6</v>
       </c>
-      <c r="K77" t="inlineStr"/>
-      <c r="L77" t="inlineStr">
+      <c r="K77" s="0" t="inlineStr"/>
+      <c r="L77" s="0" t="inlineStr">
         <is>
           <t>Straight</t>
         </is>
       </c>
-      <c r="M77" t="n">
-        <v>0</v>
-      </c>
-      <c r="N77" t="n">
-        <v>0</v>
-      </c>
-      <c r="O77" t="n">
+      <c r="M77" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N77" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O77" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="78">
-      <c r="B78" t="n">
+      <c r="B78" s="0" t="n">
         <v>75</v>
       </c>
-      <c r="C78" t="inlineStr">
+      <c r="C78" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_top_down_07</t>
         </is>
       </c>
-      <c r="D78" t="inlineStr">
+      <c r="D78" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_top_down</t>
         </is>
       </c>
-      <c r="E78" t="n">
+      <c r="E78" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="F78" t="inlineStr">
+      <c r="F78" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G78" t="n">
-        <v>1</v>
-      </c>
-      <c r="H78" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I78" t="n">
+      <c r="G78" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H78" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I78" s="0" t="n">
         <v>-0.7</v>
       </c>
-      <c r="J78" t="n">
+      <c r="J78" s="0" t="n">
         <v>7.6</v>
       </c>
-      <c r="K78" t="inlineStr"/>
-      <c r="L78" t="inlineStr">
+      <c r="K78" s="0" t="inlineStr"/>
+      <c r="L78" s="0" t="inlineStr">
         <is>
           <t>Straight</t>
         </is>
       </c>
-      <c r="M78" t="n">
-        <v>0</v>
-      </c>
-      <c r="N78" t="n">
-        <v>0</v>
-      </c>
-      <c r="O78" t="n">
+      <c r="M78" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N78" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O78" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="79">
-      <c r="B79" t="n">
+      <c r="B79" s="0" t="n">
         <v>76</v>
       </c>
-      <c r="C79" t="inlineStr">
+      <c r="C79" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_top_down_08</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr">
+      <c r="D79" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_top_down</t>
         </is>
       </c>
-      <c r="E79" t="n">
+      <c r="E79" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="F79" t="inlineStr">
+      <c r="F79" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G79" t="n">
-        <v>1</v>
-      </c>
-      <c r="H79" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I79" t="n">
+      <c r="G79" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H79" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I79" s="0" t="n">
         <v>0.7</v>
       </c>
-      <c r="J79" t="n">
+      <c r="J79" s="0" t="n">
         <v>7.6</v>
       </c>
-      <c r="K79" t="inlineStr"/>
-      <c r="L79" t="inlineStr">
+      <c r="K79" s="0" t="inlineStr"/>
+      <c r="L79" s="0" t="inlineStr">
         <is>
           <t>Straight</t>
         </is>
       </c>
-      <c r="M79" t="n">
-        <v>0</v>
-      </c>
-      <c r="N79" t="n">
-        <v>0</v>
-      </c>
-      <c r="O79" t="n">
+      <c r="M79" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N79" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O79" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="80">
-      <c r="B80" t="n">
+      <c r="B80" s="0" t="n">
         <v>77</v>
       </c>
-      <c r="C80" t="inlineStr">
+      <c r="C80" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_top_down_09</t>
         </is>
       </c>
-      <c r="D80" t="inlineStr">
+      <c r="D80" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_top_down</t>
         </is>
       </c>
-      <c r="E80" t="n">
+      <c r="E80" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="F80" t="inlineStr">
+      <c r="F80" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G80" t="n">
-        <v>1</v>
-      </c>
-      <c r="H80" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I80" t="n">
+      <c r="G80" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H80" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I80" s="0" t="n">
         <v>-0.7</v>
       </c>
-      <c r="J80" t="n">
+      <c r="J80" s="0" t="n">
         <v>6.6</v>
       </c>
-      <c r="K80" t="inlineStr"/>
-      <c r="L80" t="inlineStr">
+      <c r="K80" s="0" t="inlineStr"/>
+      <c r="L80" s="0" t="inlineStr">
         <is>
           <t>Straight</t>
         </is>
       </c>
-      <c r="M80" t="n">
-        <v>0</v>
-      </c>
-      <c r="N80" t="n">
-        <v>0</v>
-      </c>
-      <c r="O80" t="n">
+      <c r="M80" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N80" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O80" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="81">
-      <c r="B81" t="n">
+      <c r="B81" s="0" t="n">
         <v>78</v>
       </c>
-      <c r="C81" t="inlineStr">
+      <c r="C81" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_top_down_10</t>
         </is>
       </c>
-      <c r="D81" t="inlineStr">
+      <c r="D81" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_top_down</t>
         </is>
       </c>
-      <c r="E81" t="n">
+      <c r="E81" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="F81" t="inlineStr">
+      <c r="F81" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G81" t="n">
-        <v>1</v>
-      </c>
-      <c r="H81" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I81" t="n">
+      <c r="G81" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H81" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I81" s="0" t="n">
         <v>0.7</v>
       </c>
-      <c r="J81" t="n">
+      <c r="J81" s="0" t="n">
         <v>6.6</v>
       </c>
-      <c r="K81" t="inlineStr"/>
-      <c r="L81" t="inlineStr">
+      <c r="K81" s="0" t="inlineStr"/>
+      <c r="L81" s="0" t="inlineStr">
         <is>
           <t>Straight</t>
         </is>
       </c>
-      <c r="M81" t="n">
-        <v>0</v>
-      </c>
-      <c r="N81" t="n">
-        <v>0</v>
-      </c>
-      <c r="O81" t="n">
+      <c r="M81" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N81" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O81" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="82">
-      <c r="B82" t="n">
+      <c r="B82" s="0" t="n">
         <v>79</v>
       </c>
-      <c r="C82" t="inlineStr">
+      <c r="C82" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_top_down_11</t>
         </is>
       </c>
-      <c r="D82" t="inlineStr">
+      <c r="D82" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_top_down</t>
         </is>
       </c>
-      <c r="E82" t="n">
+      <c r="E82" s="0" t="n">
         <v>11</v>
       </c>
-      <c r="F82" t="inlineStr">
+      <c r="F82" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G82" t="n">
-        <v>1</v>
-      </c>
-      <c r="H82" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I82" t="n">
+      <c r="G82" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H82" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I82" s="0" t="n">
         <v>-0.7</v>
       </c>
-      <c r="J82" t="n">
+      <c r="J82" s="0" t="n">
         <v>5.6</v>
       </c>
-      <c r="K82" t="inlineStr"/>
-      <c r="L82" t="inlineStr">
+      <c r="K82" s="0" t="inlineStr"/>
+      <c r="L82" s="0" t="inlineStr">
         <is>
           <t>Straight</t>
         </is>
       </c>
-      <c r="M82" t="n">
-        <v>0</v>
-      </c>
-      <c r="N82" t="n">
-        <v>0</v>
-      </c>
-      <c r="O82" t="n">
+      <c r="M82" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N82" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O82" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="83">
-      <c r="B83" t="n">
+      <c r="B83" s="0" t="n">
         <v>80</v>
       </c>
-      <c r="C83" t="inlineStr">
+      <c r="C83" s="0" t="inlineStr">
         <is>
           <t>wave_spawn_wave_level_01_resource_top_down_12</t>
         </is>
       </c>
-      <c r="D83" t="inlineStr">
+      <c r="D83" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_top_down</t>
         </is>
       </c>
-      <c r="E83" t="n">
+      <c r="E83" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="F83" t="inlineStr">
+      <c r="F83" s="0" t="inlineStr">
         <is>
           <t>enemy_resource</t>
         </is>
       </c>
-      <c r="G83" t="n">
-        <v>1</v>
-      </c>
-      <c r="H83" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I83" t="n">
+      <c r="G83" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H83" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I83" s="0" t="n">
         <v>0.7</v>
       </c>
-      <c r="J83" t="n">
+      <c r="J83" s="0" t="n">
         <v>5.6</v>
       </c>
-      <c r="K83" t="inlineStr"/>
-      <c r="L83" t="inlineStr">
+      <c r="K83" s="0" t="inlineStr"/>
+      <c r="L83" s="0" t="inlineStr">
         <is>
           <t>Straight</t>
         </is>
       </c>
-      <c r="M83" t="n">
-        <v>0</v>
-      </c>
-      <c r="N83" t="n">
-        <v>0</v>
-      </c>
-      <c r="O83" t="n">
+      <c r="M83" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N83" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O83" s="0" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>